<commit_message>
Add evaluation notebook and restructure for EASL Summer School
- Rename main notebook to Notebook 1 (Exploration)
- Add Notebook 2: systematic LLM evaluation with RAG benchmark,
  LLM-as-judge scoring, and Gradio GUI section
- Add best-practices cells (.env, uv) to Notebook 1
- Update benchmark_data.xlsx with clinician ground truths
- Drop unused notebooks (Genial, Local LLM Inference)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmark_data.xlsx
+++ b/benchmark_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jan Clusmann\Documents\GitHub\easl_school_material\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9559DCF9-768F-49E0-AAC7-61777371EF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA834796-B028-4731-B4B1-84AFAB4035FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="1065" windowWidth="38640" windowHeight="21120" xr2:uid="{C367A0E8-6512-4812-A33E-58B20D0575AB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
   <si>
     <t>What is the working diagnosis for Ms. K.?</t>
   </si>
@@ -74,9 +74,6 @@
     <t>question</t>
   </si>
   <si>
-    <t>ground_truth</t>
-  </si>
-  <si>
     <t>model_1</t>
   </si>
   <si>
@@ -96,9 +93,6 @@
   </si>
   <si>
     <t>Yes</t>
-  </si>
-  <si>
-    <t>Either elastography or just management of comorbidieties</t>
   </si>
   <si>
     <t>&gt;= 8 kPa</t>
@@ -110,9 +104,6 @@
 • Avoiding smoking and alcohol</t>
   </si>
   <si>
-    <t>3-5% reduction</t>
-  </si>
-  <si>
     <t>type 2 diabetes, dyslipidaemia, hypertension, kidney disease, sleep apnoea, polycystic ovary syndrome</t>
   </si>
   <si>
@@ -120,6 +111,33 @@
   </si>
   <si>
     <t>Yes, Resmetirom</t>
+  </si>
+  <si>
+    <t>VCTE</t>
+  </si>
+  <si>
+    <t>weight loss, dietary changes, increased activity, less alcohol</t>
+  </si>
+  <si>
+    <t>Dyslipidaemia (Triglycerides, HDL), Obesity, (Pre-)diabetes, Hypertension</t>
+  </si>
+  <si>
+    <t>reasses Fib 4&lt;=1 year after intensified management of comorbidities</t>
+  </si>
+  <si>
+    <t>Resmetirom</t>
+  </si>
+  <si>
+    <t>ground_truth_clinician1</t>
+  </si>
+  <si>
+    <t>ground_truth_clinician2</t>
+  </si>
+  <si>
+    <t>7-10% reduction</t>
+  </si>
+  <si>
+    <t>Either elastography (VCTE) or just management of comorbidieties</t>
   </si>
 </sst>
 </file>
@@ -155,11 +173,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -494,15 +514,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33D8E1AC-06E8-4436-99C8-A5B00D008FF5}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="103.90625" customWidth="1"/>
-    <col min="3" max="3" width="50.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="3" max="3" width="55.90625" customWidth="1"/>
+    <col min="4" max="4" width="61.90625" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -510,19 +531,22 @@
         <v>10</v>
       </c>
       <c r="C1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s">
         <v>11</v>
-      </c>
-      <c r="D1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1" t="s">
-        <v>14</v>
       </c>
       <c r="F1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -530,10 +554,13 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+        <v>14</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -541,21 +568,27 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D4" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -563,10 +596,13 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -574,10 +610,13 @@
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="D6" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -585,10 +624,13 @@
         <v>4</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -596,10 +638,13 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+      <c r="D8" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -607,10 +652,13 @@
         <v>6</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -618,10 +666,13 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -629,7 +680,10 @@
         <v>8</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>